<commit_message>
fix: _load_lanc_medias le todas as sheets Geral + fix NaN posse + fix auto-loader cria DB
</commit_message>
<xml_diff>
--- a/data/medias_equipas_MULTI_LIGA.xlsx
+++ b/data/medias_equipas_MULTI_LIGA.xlsx
@@ -2634,111 +2634,41 @@
       <c r="C2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="S2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="T2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="U2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="W2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="X2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Z2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AA2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AB2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AC2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AD2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AE2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AF2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AG2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AH2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AI2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AJ2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AK2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AL2" s="2" t="n">
-        <v/>
-      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+      <c r="AC2" s="2" t="n"/>
+      <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="2" t="n"/>
+      <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
+      <c r="AJ2" s="2" t="n"/>
+      <c r="AK2" s="2" t="n"/>
+      <c r="AL2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2796,9 +2726,6 @@
       <c r="Q3" t="n">
         <v>0.5</v>
       </c>
-      <c r="R3" t="n">
-        <v/>
-      </c>
       <c r="S3" t="n">
         <v>0.52</v>
       </c>
@@ -4123,7 +4050,7 @@
         <v>0.85</v>
       </c>
       <c r="T14" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U14" s="2" t="n">
         <v>1.38</v>
@@ -10360,7 +10287,7 @@
         <v>1.62</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="T2" s="2" t="n">
         <v>3.21</v>
@@ -12651,7 +12578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL18"/>
+  <dimension ref="A1:AL21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12898,7 +12825,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.38</v>
@@ -12958,7 +12885,7 @@
         <v>8.210000000000001</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>20.71</v>
+        <v>19.82</v>
       </c>
       <c r="X2" s="2" t="n">
         <v>12.62</v>
@@ -14924,6 +14851,94 @@
       </c>
       <c r="AL18" s="2" t="n">
         <v>1.32</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PPL</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Vitoria Guimaraes</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="W19" t="n">
+        <v>19.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PPL</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Maritimo</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" s="2" t="n"/>
+      <c r="S20" s="2" t="n"/>
+      <c r="T20" s="2" t="n"/>
+      <c r="U20" s="2" t="n"/>
+      <c r="V20" s="2" t="n"/>
+      <c r="W20" s="2" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="X20" s="2" t="n"/>
+      <c r="Y20" s="2" t="n"/>
+      <c r="Z20" s="2" t="n"/>
+      <c r="AA20" s="2" t="n"/>
+      <c r="AB20" s="2" t="n"/>
+      <c r="AC20" s="2" t="n"/>
+      <c r="AD20" s="2" t="n"/>
+      <c r="AE20" s="2" t="n"/>
+      <c r="AF20" s="2" t="n"/>
+      <c r="AG20" s="2" t="n"/>
+      <c r="AH20" s="2" t="n"/>
+      <c r="AI20" s="2" t="n"/>
+      <c r="AJ20" s="2" t="n"/>
+      <c r="AK20" s="2" t="n"/>
+      <c r="AL20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PPL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Academico Viseu</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>11</v>
+      </c>
+      <c r="W21" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -16915,7 +16930,7 @@
         <v>1.6</v>
       </c>
       <c r="T16" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U16" s="2" t="n">
         <v>2.83</v>
@@ -17121,9 +17136,7 @@
       <c r="H18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n">
         <v>18.5</v>
       </c>
@@ -17148,9 +17161,7 @@
       <c r="Q18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R18" s="2" t="n">
-        <v/>
-      </c>
+      <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n">
         <v>1.99</v>
       </c>
@@ -17472,111 +17483,41 @@
       <c r="C2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="S2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="T2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="U2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="W2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="X2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="Z2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AA2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AB2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AC2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AD2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AE2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AF2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AG2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AH2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AI2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AJ2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AK2" s="2" t="n">
-        <v/>
-      </c>
-      <c r="AL2" s="2" t="n">
-        <v/>
-      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+      <c r="AC2" s="2" t="n"/>
+      <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="2" t="n"/>
+      <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
+      <c r="AJ2" s="2" t="n"/>
+      <c r="AK2" s="2" t="n"/>
+      <c r="AL2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17607,9 +17548,6 @@
       <c r="H3" t="n">
         <v>2.5</v>
       </c>
-      <c r="I3" t="n">
-        <v/>
-      </c>
       <c r="J3" t="n">
         <v>11.5</v>
       </c>
@@ -17633,9 +17571,6 @@
       </c>
       <c r="Q3" t="n">
         <v>2</v>
-      </c>
-      <c r="R3" t="n">
-        <v/>
       </c>
       <c r="S3" t="n">
         <v>0.8100000000000001</v>
@@ -18207,9 +18142,7 @@
       <c r="H8" s="2" t="n">
         <v>2.17</v>
       </c>
-      <c r="I8" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n">
         <v>19.42</v>
       </c>
@@ -24219,9 +24152,7 @@
       <c r="H18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n">
         <v>21.67</v>
       </c>
@@ -24338,9 +24269,6 @@
       </c>
       <c r="H19" t="n">
         <v>3</v>
-      </c>
-      <c r="I19" t="n">
-        <v/>
       </c>
       <c r="J19" t="n">
         <v>24.5</v>

</xml_diff>